<commit_message>
Completar diccionario y agregar draft de lstm
</commit_message>
<xml_diff>
--- a/inputs/diccionario.xlsx
+++ b/inputs/diccionario.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eaneg\OneDrive\Desktop\Datos TP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Eugenio\Maestria\Series Temporales\series_temporales_2025\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54443985-89BE-4325-9678-F940C7FFB768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40425F3B-61C8-4E68-BDFD-0DA4A9752E49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="85">
   <si>
     <t>fecha</t>
   </si>
@@ -252,15 +252,60 @@
   <si>
     <t>UVA</t>
   </si>
+  <si>
+    <t>m1</t>
+  </si>
+  <si>
+    <t>Agregado monetario que comprende, en la Argentina, circulante en poder del público más cuentas corrientes en pesos del sector público y privado no financiero. </t>
+  </si>
+  <si>
+    <t>m2</t>
+  </si>
+  <si>
+    <t>Medios de pago, comprende circulante en poder del público más depósitos a la vista en pesos del sector público y privado no financiero. </t>
+  </si>
+  <si>
+    <t>m3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agregado monetario amplio, comprende circulante en poder del público más total de depósitos en pesos del sector público y privado no financiero. </t>
+  </si>
+  <si>
+    <t>inflacion</t>
+  </si>
+  <si>
+    <t>Tasa de variación mensual</t>
+  </si>
+  <si>
+    <t>Elaboracion propia en base a BCRA</t>
+  </si>
+  <si>
+    <t>Inflación mensual</t>
+  </si>
+  <si>
+    <t>rem</t>
+  </si>
+  <si>
+    <t>Inflación esperada - REM próximos 12 meses - MEDIANA (variación en i.a)</t>
+  </si>
+  <si>
+    <t>Tasa de variación anual</t>
+  </si>
+  <si>
+    <t>prestamos_privados_en_pesos_ars</t>
+  </si>
+  <si>
+    <t>Stock de prestamos en pesos al sector privado</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="172" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -272,6 +317,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -298,16 +349,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -17544,7 +17596,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D68D9661-D5F8-4698-9487-A24691442B2A}">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
@@ -17977,6 +18029,108 @@
         <v>46</v>
       </c>
     </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>70</v>
+      </c>
+      <c r="B26" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" t="s">
+        <v>20</v>
+      </c>
+      <c r="D26" t="s">
+        <v>71</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>72</v>
+      </c>
+      <c r="B27" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" t="s">
+        <v>20</v>
+      </c>
+      <c r="D27" t="s">
+        <v>73</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>74</v>
+      </c>
+      <c r="B28" t="s">
+        <v>59</v>
+      </c>
+      <c r="C28" t="s">
+        <v>20</v>
+      </c>
+      <c r="D28" t="s">
+        <v>75</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>76</v>
+      </c>
+      <c r="B29" t="s">
+        <v>77</v>
+      </c>
+      <c r="C29" t="s">
+        <v>25</v>
+      </c>
+      <c r="D29" t="s">
+        <v>79</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>80</v>
+      </c>
+      <c r="B30" t="s">
+        <v>82</v>
+      </c>
+      <c r="C30" t="s">
+        <v>25</v>
+      </c>
+      <c r="D30" t="s">
+        <v>81</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>83</v>
+      </c>
+      <c r="B31" t="s">
+        <v>59</v>
+      </c>
+      <c r="C31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" t="s">
+        <v>84</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" xr:uid="{367FD9AC-ED1F-4BF3-8464-A874C9BF1185}"/>
@@ -17985,6 +18139,9 @@
     <hyperlink ref="E9" r:id="rId4" xr:uid="{570D3B3F-B1C2-4459-A684-E7EE4C8EA780}"/>
     <hyperlink ref="E8" r:id="rId5" xr:uid="{AADE2B87-8679-4A1A-AFD1-91980FA8EC08}"/>
     <hyperlink ref="E7" r:id="rId6" xr:uid="{0574CB13-C3FA-4963-9589-C7E5AD7B791E}"/>
+    <hyperlink ref="E29" r:id="rId7" xr:uid="{C0365983-E341-4415-8B33-003D3D04E6BF}"/>
+    <hyperlink ref="E30" r:id="rId8" xr:uid="{FED48BAD-8C63-476A-80B7-A83938422758}"/>
+    <hyperlink ref="E31" r:id="rId9" xr:uid="{94DCFB4E-22E7-4981-BAE5-80A634946772}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>